<commit_message>
BOS 589282: leave COO as not stated (no origin in any document)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TiaFcfbZGSaW3eVMooPrNx
</commit_message>
<xml_diff>
--- a/output/HS_Code_Summary_BOS_Automotive_589282.xlsx
+++ b/output/HS_Code_Summary_BOS_Automotive_589282.xlsx
@@ -600,7 +600,7 @@
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>neuvedeno na faktuře (odeslání MX)</t>
+          <t>neuvedeno</t>
         </is>
       </c>
       <c r="E6" s="5" t="n">
@@ -987,7 +987,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Pole „Ursprungsland“ na faktuře je prázdné; B/L „Point and country of origin“ také prázdné. Odesláno z MX – COO potvrdit.</t>
+          <t>Pole „Ursprungsland“ na faktuře je prázdné; B/L „Point and country of origin“ také prázdné. Země původu není uvedena v žádném dokladu – v souhrnu ponecháno „neuvedeno“ (MX se nepředpokládá). Nutno doložit od BOS Irapuato.</t>
         </is>
       </c>
     </row>
@@ -1008,7 +1008,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>→ Bez prohlášení o původu platí konvenční clo (7326 90 98: 2,7 %). Pokud je zboží mexického původu, lze vyžádat prohlášení o původu dle dohody EU–Mexiko pro preferenční 0 %.</t>
+          <t>→ Bez prohlášení o původu platí konvenční clo (7326 90 98: 2,7 %). Pokud by odesílatel doložil mexický původ, lze vyžádat prohlášení o původu dle dohody EU–Mexiko pro preferenční 0 %.</t>
         </is>
       </c>
     </row>

</xml_diff>